<commit_message>
Weekly data update: camera_events.xlsx
</commit_message>
<xml_diff>
--- a/camera_events.xlsx
+++ b/camera_events.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Shared drives\Synergy Safety Group\DEN\Dashboard\Weekly Dashboards\Curtis-Garage-Wrecker-Service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3538CBBB-468A-4A06-848D-F0CE914019F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{07787563-9BCD-42E0-8032-BBAE9E4F8AEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3240" yWindow="3240" windowWidth="43200" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DRIVE-ALERTS" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10600" uniqueCount="4363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11035" uniqueCount="4550">
   <si>
     <t>DRIVE ALERTS</t>
   </si>
@@ -13006,6 +13006,9 @@
     <t>39.523525, -86.810090</t>
   </si>
   <si>
+    <t>06/21/26 22:24 EDT</t>
+  </si>
+  <si>
     <t>06/19/26 07:23 EDT</t>
   </si>
   <si>
@@ -13069,6 +13072,9 @@
     <t>39.545850, -86.729060</t>
   </si>
   <si>
+    <t>06/21/26 22:25 EDT</t>
+  </si>
+  <si>
     <t>06/20/26 21:43 EDT</t>
   </si>
   <si>
@@ -13081,6 +13087,9 @@
     <t>39.530563, -86.802990</t>
   </si>
   <si>
+    <t>06/22/26 12:10 EDT</t>
+  </si>
+  <si>
     <t>06/20/26 21:54 EDT</t>
   </si>
   <si>
@@ -13099,16 +13108,568 @@
     <t>39.528000, -86.877240</t>
   </si>
   <si>
+    <t>06/21/26 22:26 EDT</t>
+  </si>
+  <si>
     <t>06/21/26 05:14 EDT</t>
   </si>
   <si>
     <t>39.505913, -86.549560</t>
   </si>
   <si>
+    <t>06/21/26 22:27 EDT</t>
+  </si>
+  <si>
     <t>06/21/26 05:15 EDT</t>
   </si>
   <si>
     <t>39.506153, -86.563550</t>
+  </si>
+  <si>
+    <t>06/22/26 05:50 EDT</t>
+  </si>
+  <si>
+    <t>39.564800, -86.608060</t>
+  </si>
+  <si>
+    <t>06/22/26 12:34 EDT</t>
+  </si>
+  <si>
+    <t>06/22/26 13:40 EDT</t>
+  </si>
+  <si>
+    <t>06/22/26 07:56 EDT</t>
+  </si>
+  <si>
+    <t>39.558025, -86.743190</t>
+  </si>
+  <si>
+    <t>06/23/26 08:28 EDT</t>
+  </si>
+  <si>
+    <t>06/22/26 08:06 EDT</t>
+  </si>
+  <si>
+    <t>39.579400, -86.638500</t>
+  </si>
+  <si>
+    <t>06/22/26 10:10 EDT</t>
+  </si>
+  <si>
+    <t>39.567978, -86.633410</t>
+  </si>
+  <si>
+    <t>06/23/26 08:38 EDT</t>
+  </si>
+  <si>
+    <t>06/22/26 11:06 EDT</t>
+  </si>
+  <si>
+    <t>39.569435, -86.632100</t>
+  </si>
+  <si>
+    <t>06/22/26 11:15 EDT</t>
+  </si>
+  <si>
+    <t>39.579086, -86.540660</t>
+  </si>
+  <si>
+    <t>06/22/26 12:12 EDT</t>
+  </si>
+  <si>
+    <t>1.5mi NE of Plainfield IN</t>
+  </si>
+  <si>
+    <t>39.712353, -86.354910</t>
+  </si>
+  <si>
+    <t>06/22/26 12:22 EDT</t>
+  </si>
+  <si>
+    <t>39.637640, -86.433650</t>
+  </si>
+  <si>
+    <t>06/22/26 13:06 EDT</t>
+  </si>
+  <si>
+    <t>11.3mi S of Greencastle IN</t>
+  </si>
+  <si>
+    <t>39.486122, -86.785010</t>
+  </si>
+  <si>
+    <t>06/22/26 13:21 EDT</t>
+  </si>
+  <si>
+    <t>39.568027, -86.633610</t>
+  </si>
+  <si>
+    <t>06/23/26 08:29 EDT</t>
+  </si>
+  <si>
+    <t>06/22/26 15:01 EDT</t>
+  </si>
+  <si>
+    <t>39.580917, -86.591900</t>
+  </si>
+  <si>
+    <t>06/23/26 08:45 EDT</t>
+  </si>
+  <si>
+    <t>06/22/26 15:59 EDT</t>
+  </si>
+  <si>
+    <t>1.1mi N of Plainfield IN</t>
+  </si>
+  <si>
+    <t>39.711790, -86.370090</t>
+  </si>
+  <si>
+    <t>06/22/26 16:32 EDT</t>
+  </si>
+  <si>
+    <t>5.5mi SE of Brazil IN</t>
+  </si>
+  <si>
+    <t>39.466908, -87.050340</t>
+  </si>
+  <si>
+    <t>06/23/26 08:33 EDT</t>
+  </si>
+  <si>
+    <t>06/22/26 17:22 EDT</t>
+  </si>
+  <si>
+    <t>2.6mi NW of Terre Haute IN</t>
+  </si>
+  <si>
+    <t>39.496758, -87.401726</t>
+  </si>
+  <si>
+    <t>06/23/26 08:34 EDT</t>
+  </si>
+  <si>
+    <t>06/22/26 18:27 EDT</t>
+  </si>
+  <si>
+    <t>39.557335, -86.674730</t>
+  </si>
+  <si>
+    <t>06/22/26 20:19 EDT</t>
+  </si>
+  <si>
+    <t>39.564840, -86.615990</t>
+  </si>
+  <si>
+    <t>06/22/26 20:24 EDT</t>
+  </si>
+  <si>
+    <t>39.535660, -86.577260</t>
+  </si>
+  <si>
+    <t>06/23/26 08:14 EDT</t>
+  </si>
+  <si>
+    <t>39.590030, -86.628910</t>
+  </si>
+  <si>
+    <t>06/23/26 09:38 EDT</t>
+  </si>
+  <si>
+    <t>2.9mi SE of Plainfield IN</t>
+  </si>
+  <si>
+    <t>39.677710, -86.322730</t>
+  </si>
+  <si>
+    <t>06/23/26 11:06 EDT</t>
+  </si>
+  <si>
+    <t>39.647568, -86.409190</t>
+  </si>
+  <si>
+    <t>06/24/26 08:09 EDT</t>
+  </si>
+  <si>
+    <t>06/23/26 12:25 EDT</t>
+  </si>
+  <si>
+    <t>3.2mi E of Plainfield IN</t>
+  </si>
+  <si>
+    <t>39.692060, -86.310875</t>
+  </si>
+  <si>
+    <t>06/24/26 08:18 EDT</t>
+  </si>
+  <si>
+    <t>06/24/26 08:21 EDT</t>
+  </si>
+  <si>
+    <t>06/23/26 14:53 EDT</t>
+  </si>
+  <si>
+    <t>39.520927, -86.564060</t>
+  </si>
+  <si>
+    <t>06/23/26 14:57 EDT</t>
+  </si>
+  <si>
+    <t>2mi N of Greenfield IN</t>
+  </si>
+  <si>
+    <t>39.820870, -85.787420</t>
+  </si>
+  <si>
+    <t>06/23/26 15:07 EDT</t>
+  </si>
+  <si>
+    <t>3.4mi W of Cumberland IN</t>
+  </si>
+  <si>
+    <t>39.801020, -86.005430</t>
+  </si>
+  <si>
+    <t>06/23/26 15:21 EDT</t>
+  </si>
+  <si>
+    <t>1.8mi SW of Indianapolis IN</t>
+  </si>
+  <si>
+    <t>39.753600, -86.159990</t>
+  </si>
+  <si>
+    <t>06/23/26 15:22 EDT</t>
+  </si>
+  <si>
+    <t>39.754440, -86.180130</t>
+  </si>
+  <si>
+    <t>06/23/26 16:25 EDT</t>
+  </si>
+  <si>
+    <t>4.5mi NW of Mooresville IN</t>
+  </si>
+  <si>
+    <t>39.632980, -86.442340</t>
+  </si>
+  <si>
+    <t>06/23/26 18:57 EDT</t>
+  </si>
+  <si>
+    <t>5.9mi NE of Greencastle IN</t>
+  </si>
+  <si>
+    <t>39.683000, -86.743390</t>
+  </si>
+  <si>
+    <t>06/24/26 06:32 EDT</t>
+  </si>
+  <si>
+    <t>39.634876, -86.649820</t>
+  </si>
+  <si>
+    <t>06/24/26 08:00 EDT</t>
+  </si>
+  <si>
+    <t>06/24/26 06:39 EDT</t>
+  </si>
+  <si>
+    <t>39.564530, -86.643040</t>
+  </si>
+  <si>
+    <t>06/24/26 06:46 EDT</t>
+  </si>
+  <si>
+    <t>39.558758, -86.666000</t>
+  </si>
+  <si>
+    <t>06/24/26 08:29 EDT</t>
+  </si>
+  <si>
+    <t>39.528008, -86.877240</t>
+  </si>
+  <si>
+    <t>06/24/26 17:31 EDT</t>
+  </si>
+  <si>
+    <t>39.557003, -86.677830</t>
+  </si>
+  <si>
+    <t>06/24/26 22:51 EDT</t>
+  </si>
+  <si>
+    <t>39.565025, -86.631980</t>
+  </si>
+  <si>
+    <t>06/25/26 00:00 EDT</t>
+  </si>
+  <si>
+    <t>39.533497, -86.804855</t>
+  </si>
+  <si>
+    <t>06/25/26 07:36 EDT</t>
+  </si>
+  <si>
+    <t>06/25/26 00:01 EDT</t>
+  </si>
+  <si>
+    <t>39.529682, -86.802280</t>
+  </si>
+  <si>
+    <t>06/25/26 07:54 EDT</t>
+  </si>
+  <si>
+    <t>39.511906, -86.641945</t>
+  </si>
+  <si>
+    <t>06/25/26 21:15 EDT</t>
+  </si>
+  <si>
+    <t>06/25/26 09:16 EDT</t>
+  </si>
+  <si>
+    <t>39.568317, -86.633630</t>
+  </si>
+  <si>
+    <t>06/25/26 21:10 EDT</t>
+  </si>
+  <si>
+    <t>06/25/26 14:45 EDT</t>
+  </si>
+  <si>
+    <t>39.571300, -86.628340</t>
+  </si>
+  <si>
+    <t>06/25/26 15:18 EDT</t>
+  </si>
+  <si>
+    <t>39.549034, -86.717790</t>
+  </si>
+  <si>
+    <t>06/25/26 15:25 EDT</t>
+  </si>
+  <si>
+    <t>39.684550, -86.462260</t>
+  </si>
+  <si>
+    <t>06/25/26 16:24 EDT</t>
+  </si>
+  <si>
+    <t>5mi W of Mooresville IN</t>
+  </si>
+  <si>
+    <t>39.622900, -86.458210</t>
+  </si>
+  <si>
+    <t>06/25/26 16:30 EDT</t>
+  </si>
+  <si>
+    <t>39.585255, -86.577410</t>
+  </si>
+  <si>
+    <t>06/25/26 21:21 EDT</t>
+  </si>
+  <si>
+    <t>06/25/26 21:26 EDT</t>
+  </si>
+  <si>
+    <t>06/25/26 17:26 EDT</t>
+  </si>
+  <si>
+    <t>39.630310, -86.669716</t>
+  </si>
+  <si>
+    <t>06/26/26 06:54 EDT</t>
+  </si>
+  <si>
+    <t>39.568172, -86.632170</t>
+  </si>
+  <si>
+    <t>06/26/26 07:35 EDT</t>
+  </si>
+  <si>
+    <t>06/26/26 07:37 EDT</t>
+  </si>
+  <si>
+    <t>39.710236, -86.669850</t>
+  </si>
+  <si>
+    <t>06/26/26 07:52 EDT</t>
+  </si>
+  <si>
+    <t>39.579350, -86.631910</t>
+  </si>
+  <si>
+    <t>06/26/26 12:07 EDT</t>
+  </si>
+  <si>
+    <t>39.589073, -86.559950</t>
+  </si>
+  <si>
+    <t>2.6mi W of Plainfield IN</t>
+  </si>
+  <si>
+    <t>39.682827, -86.418470</t>
+  </si>
+  <si>
+    <t>06/26/26 12:11 EDT</t>
+  </si>
+  <si>
+    <t>39.619995, -86.462290</t>
+  </si>
+  <si>
+    <t>06/26/26 12:32 EDT</t>
+  </si>
+  <si>
+    <t>3.2mi S of Beech Grove IN</t>
+  </si>
+  <si>
+    <t>39.670200, -86.096280</t>
+  </si>
+  <si>
+    <t>06/26/26 12:49 EDT</t>
+  </si>
+  <si>
+    <t>2.7mi NE of Greenwood IN</t>
+  </si>
+  <si>
+    <t>39.633102, -86.077990</t>
+  </si>
+  <si>
+    <t>06/26/26 13:07 EDT</t>
+  </si>
+  <si>
+    <t>6.2mi E of Plainfield IN</t>
+  </si>
+  <si>
+    <t>39.696910, -86.254166</t>
+  </si>
+  <si>
+    <t>06/26/26 13:30 EDT</t>
+  </si>
+  <si>
+    <t>39.552074, -86.706970</t>
+  </si>
+  <si>
+    <t>06/26/26 13:35 EDT</t>
+  </si>
+  <si>
+    <t>39.533030, -86.819405</t>
+  </si>
+  <si>
+    <t>06/26/26 13:37 EDT</t>
+  </si>
+  <si>
+    <t>39.531006, -86.861275</t>
+  </si>
+  <si>
+    <t>06/26/26 13:38 EDT</t>
+  </si>
+  <si>
+    <t>39.529263, -86.869040</t>
+  </si>
+  <si>
+    <t>06/26/26 14:42 EDT</t>
+  </si>
+  <si>
+    <t>6.5mi W of Brazil IN</t>
+  </si>
+  <si>
+    <t>39.520927, -87.245400</t>
+  </si>
+  <si>
+    <t>06/26/26 15:22 EDT</t>
+  </si>
+  <si>
+    <t>39.569466, -86.632110</t>
+  </si>
+  <si>
+    <t>06/26/26 19:39 EDT</t>
+  </si>
+  <si>
+    <t>39.499370, -86.661660</t>
+  </si>
+  <si>
+    <t>06/27/26 12:17 EDT</t>
+  </si>
+  <si>
+    <t>5.2mi SW of Carmel IN</t>
+  </si>
+  <si>
+    <t>39.923855, -86.228430</t>
+  </si>
+  <si>
+    <t>06/27/26 12:30 EDT</t>
+  </si>
+  <si>
+    <t>6.3mi SE of Zionsville IN</t>
+  </si>
+  <si>
+    <t>39.909880, -86.260445</t>
+  </si>
+  <si>
+    <t>06/27/26 12:31 EDT</t>
+  </si>
+  <si>
+    <t>6.4mi SE of Zionsville IN</t>
+  </si>
+  <si>
+    <t>39.909160, -86.259920</t>
+  </si>
+  <si>
+    <t>06/27/26 12:56 EDT</t>
+  </si>
+  <si>
+    <t>39.533630, -86.789100</t>
+  </si>
+  <si>
+    <t>06/27/26 20:31 EDT</t>
+  </si>
+  <si>
+    <t>39.595627, -86.530780</t>
+  </si>
+  <si>
+    <t>06/27/26 20:41 EDT</t>
+  </si>
+  <si>
+    <t>39.675520, -86.351290</t>
+  </si>
+  <si>
+    <t>06/27/26 22:21 EDT</t>
+  </si>
+  <si>
+    <t>39.556526, -86.646355</t>
+  </si>
+  <si>
+    <t>06/28/26 02:50 EDT</t>
+  </si>
+  <si>
+    <t>39.525684, -86.809930</t>
+  </si>
+  <si>
+    <t>06/28/26 03:08 EDT</t>
+  </si>
+  <si>
+    <t>39.610016, -86.490870</t>
+  </si>
+  <si>
+    <t>06/28/26 04:10 EDT</t>
+  </si>
+  <si>
+    <t>4.1mi N of Terre Haute IN</t>
+  </si>
+  <si>
+    <t>39.523970, -87.360310</t>
+  </si>
+  <si>
+    <t>06/28/26 04:13 EDT</t>
+  </si>
+  <si>
+    <t>4.6mi N of Terre Haute IN</t>
+  </si>
+  <si>
+    <t>39.532330, -87.369840</t>
   </si>
 </sst>
 </file>
@@ -13470,12 +14031,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N1736"/>
+  <dimension ref="A1:N1807"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="14" width="15" customWidth="1"/>
+    <col min="1" max="14" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -73158,19 +73717,25 @@
       <c r="G1719" s="3" t="s">
         <v>4327</v>
       </c>
-      <c r="H1719" s="3"/>
+      <c r="H1719" s="3" t="s">
+        <v>276</v>
+      </c>
       <c r="I1719" s="3"/>
       <c r="J1719" s="3"/>
       <c r="K1719" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1719" s="3"/>
-      <c r="M1719" s="3"/>
+        <v>80</v>
+      </c>
+      <c r="L1719" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1719" s="3" t="s">
+        <v>4328</v>
+      </c>
       <c r="N1719" s="3"/>
     </row>
     <row r="1720" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1720" s="3" t="s">
-        <v>4328</v>
+        <v>4329</v>
       </c>
       <c r="B1720" s="3"/>
       <c r="C1720" s="3">
@@ -73186,7 +73751,7 @@
         <v>3231</v>
       </c>
       <c r="G1720" s="3" t="s">
-        <v>4329</v>
+        <v>4330</v>
       </c>
       <c r="H1720" s="3"/>
       <c r="I1720" s="3">
@@ -73202,7 +73767,7 @@
     </row>
     <row r="1721" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1721" s="3" t="s">
-        <v>4330</v>
+        <v>4331</v>
       </c>
       <c r="B1721" s="3"/>
       <c r="C1721" s="3">
@@ -73218,7 +73783,7 @@
         <v>531</v>
       </c>
       <c r="G1721" s="3" t="s">
-        <v>4331</v>
+        <v>4332</v>
       </c>
       <c r="H1721" s="3"/>
       <c r="I1721" s="3">
@@ -73234,7 +73799,7 @@
     </row>
     <row r="1722" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1722" s="3" t="s">
-        <v>4332</v>
+        <v>4333</v>
       </c>
       <c r="B1722" s="3"/>
       <c r="C1722" s="3">
@@ -73250,7 +73815,7 @@
         <v>516</v>
       </c>
       <c r="G1722" s="3" t="s">
-        <v>4333</v>
+        <v>4334</v>
       </c>
       <c r="H1722" s="3"/>
       <c r="I1722" s="3">
@@ -73268,7 +73833,7 @@
     </row>
     <row r="1723" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1723" s="3" t="s">
-        <v>4334</v>
+        <v>4335</v>
       </c>
       <c r="B1723" s="3"/>
       <c r="C1723" s="3">
@@ -73284,7 +73849,7 @@
         <v>522</v>
       </c>
       <c r="G1723" s="3" t="s">
-        <v>4335</v>
+        <v>4336</v>
       </c>
       <c r="H1723" s="3"/>
       <c r="I1723" s="3">
@@ -73302,7 +73867,7 @@
     </row>
     <row r="1724" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1724" s="3" t="s">
-        <v>4336</v>
+        <v>4337</v>
       </c>
       <c r="B1724" s="3"/>
       <c r="C1724" s="3">
@@ -73318,7 +73883,7 @@
         <v>492</v>
       </c>
       <c r="G1724" s="3" t="s">
-        <v>4337</v>
+        <v>4338</v>
       </c>
       <c r="H1724" s="3"/>
       <c r="I1724" s="3">
@@ -73336,7 +73901,7 @@
     </row>
     <row r="1725" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1725" s="3" t="s">
-        <v>4338</v>
+        <v>4339</v>
       </c>
       <c r="B1725" s="3"/>
       <c r="C1725" s="3">
@@ -73352,7 +73917,7 @@
         <v>3114</v>
       </c>
       <c r="G1725" s="3" t="s">
-        <v>4339</v>
+        <v>4340</v>
       </c>
       <c r="H1725" s="3"/>
       <c r="I1725" s="3">
@@ -73370,7 +73935,7 @@
     </row>
     <row r="1726" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1726" s="3" t="s">
-        <v>4340</v>
+        <v>4341</v>
       </c>
       <c r="B1726" s="3"/>
       <c r="C1726" s="3">
@@ -73386,7 +73951,7 @@
         <v>1968</v>
       </c>
       <c r="G1726" s="3" t="s">
-        <v>4341</v>
+        <v>4342</v>
       </c>
       <c r="H1726" s="3"/>
       <c r="I1726" s="3">
@@ -73404,7 +73969,7 @@
     </row>
     <row r="1727" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1727" s="3" t="s">
-        <v>4342</v>
+        <v>4343</v>
       </c>
       <c r="B1727" s="3"/>
       <c r="C1727" s="3">
@@ -73420,7 +73985,7 @@
         <v>274</v>
       </c>
       <c r="G1727" s="3" t="s">
-        <v>4343</v>
+        <v>4344</v>
       </c>
       <c r="H1727" s="3"/>
       <c r="I1727" s="3">
@@ -73436,7 +74001,7 @@
     </row>
     <row r="1728" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1728" s="3" t="s">
-        <v>4344</v>
+        <v>4345</v>
       </c>
       <c r="B1728" s="3"/>
       <c r="C1728" s="3">
@@ -73449,10 +74014,10 @@
         <v>17</v>
       </c>
       <c r="F1728" s="3" t="s">
-        <v>4345</v>
+        <v>4346</v>
       </c>
       <c r="G1728" s="3" t="s">
-        <v>4346</v>
+        <v>4347</v>
       </c>
       <c r="H1728" s="3"/>
       <c r="I1728" s="3">
@@ -73470,7 +74035,7 @@
     </row>
     <row r="1729" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1729" s="3" t="s">
-        <v>4347</v>
+        <v>4348</v>
       </c>
       <c r="B1729" s="3"/>
       <c r="C1729" s="3">
@@ -73486,23 +74051,29 @@
         <v>637</v>
       </c>
       <c r="G1729" s="3" t="s">
-        <v>4348</v>
-      </c>
-      <c r="H1729" s="3"/>
+        <v>4349</v>
+      </c>
+      <c r="H1729" s="3" t="s">
+        <v>276</v>
+      </c>
       <c r="I1729" s="3">
         <v>42</v>
       </c>
       <c r="J1729" s="3"/>
       <c r="K1729" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1729" s="3"/>
-      <c r="M1729" s="3"/>
+        <v>80</v>
+      </c>
+      <c r="L1729" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1729" s="3" t="s">
+        <v>4350</v>
+      </c>
       <c r="N1729" s="3"/>
     </row>
     <row r="1730" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1730" s="3" t="s">
-        <v>4349</v>
+        <v>4351</v>
       </c>
       <c r="B1730" s="3"/>
       <c r="C1730" s="3">
@@ -73518,21 +74089,27 @@
         <v>270</v>
       </c>
       <c r="G1730" s="3" t="s">
-        <v>4350</v>
-      </c>
-      <c r="H1730" s="3"/>
+        <v>4352</v>
+      </c>
+      <c r="H1730" s="3" t="s">
+        <v>276</v>
+      </c>
       <c r="I1730" s="3"/>
       <c r="J1730" s="3"/>
       <c r="K1730" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1730" s="3"/>
-      <c r="M1730" s="3"/>
+        <v>80</v>
+      </c>
+      <c r="L1730" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1730" s="3" t="s">
+        <v>4350</v>
+      </c>
       <c r="N1730" s="3"/>
     </row>
     <row r="1731" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1731" s="3" t="s">
-        <v>4351</v>
+        <v>4353</v>
       </c>
       <c r="B1731" s="3"/>
       <c r="C1731" s="3">
@@ -73548,23 +74125,29 @@
         <v>215</v>
       </c>
       <c r="G1731" s="3" t="s">
-        <v>4352</v>
-      </c>
-      <c r="H1731" s="3"/>
+        <v>4354</v>
+      </c>
+      <c r="H1731" s="3" t="s">
+        <v>276</v>
+      </c>
       <c r="I1731" s="3">
         <v>8</v>
       </c>
       <c r="J1731" s="3"/>
       <c r="K1731" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1731" s="3"/>
-      <c r="M1731" s="3"/>
+        <v>80</v>
+      </c>
+      <c r="L1731" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1731" s="3" t="s">
+        <v>4355</v>
+      </c>
       <c r="N1731" s="3"/>
     </row>
     <row r="1732" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1732" s="3" t="s">
-        <v>4353</v>
+        <v>4356</v>
       </c>
       <c r="B1732" s="3"/>
       <c r="C1732" s="3">
@@ -73580,7 +74163,7 @@
         <v>745</v>
       </c>
       <c r="G1732" s="3" t="s">
-        <v>4354</v>
+        <v>4357</v>
       </c>
       <c r="H1732" s="3"/>
       <c r="I1732" s="3">
@@ -73596,7 +74179,7 @@
     </row>
     <row r="1733" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1733" s="3" t="s">
-        <v>4355</v>
+        <v>4358</v>
       </c>
       <c r="B1733" s="3"/>
       <c r="C1733" s="3">
@@ -73612,7 +74195,7 @@
         <v>637</v>
       </c>
       <c r="G1733" s="3" t="s">
-        <v>4356</v>
+        <v>4359</v>
       </c>
       <c r="H1733" s="3"/>
       <c r="I1733" s="3">
@@ -73628,7 +74211,7 @@
     </row>
     <row r="1734" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1734" s="3" t="s">
-        <v>4357</v>
+        <v>4360</v>
       </c>
       <c r="B1734" s="3"/>
       <c r="C1734" s="3">
@@ -73644,23 +74227,29 @@
         <v>218</v>
       </c>
       <c r="G1734" s="3" t="s">
-        <v>4358</v>
-      </c>
-      <c r="H1734" s="3"/>
+        <v>4361</v>
+      </c>
+      <c r="H1734" s="3" t="s">
+        <v>276</v>
+      </c>
       <c r="I1734" s="3">
         <v>32</v>
       </c>
       <c r="J1734" s="3"/>
       <c r="K1734" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1734" s="3"/>
-      <c r="M1734" s="3"/>
+        <v>80</v>
+      </c>
+      <c r="L1734" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1734" s="3" t="s">
+        <v>4362</v>
+      </c>
       <c r="N1734" s="3"/>
     </row>
     <row r="1735" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1735" s="3" t="s">
-        <v>4359</v>
+        <v>4363</v>
       </c>
       <c r="B1735" s="3"/>
       <c r="C1735" s="3">
@@ -73676,23 +74265,29 @@
         <v>118</v>
       </c>
       <c r="G1735" s="3" t="s">
-        <v>4360</v>
-      </c>
-      <c r="H1735" s="3"/>
+        <v>4364</v>
+      </c>
+      <c r="H1735" s="3" t="s">
+        <v>276</v>
+      </c>
       <c r="I1735" s="3">
         <v>33</v>
       </c>
       <c r="J1735" s="3"/>
       <c r="K1735" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1735" s="3"/>
-      <c r="M1735" s="3"/>
+        <v>80</v>
+      </c>
+      <c r="L1735" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1735" s="3" t="s">
+        <v>4365</v>
+      </c>
       <c r="N1735" s="3"/>
     </row>
     <row r="1736" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1736" s="3" t="s">
-        <v>4361</v>
+        <v>4366</v>
       </c>
       <c r="B1736" s="3"/>
       <c r="C1736" s="3">
@@ -73708,7 +74303,7 @@
         <v>159</v>
       </c>
       <c r="G1736" s="3" t="s">
-        <v>4362</v>
+        <v>4367</v>
       </c>
       <c r="H1736" s="3"/>
       <c r="I1736" s="3">
@@ -73721,6 +74316,2420 @@
       <c r="L1736" s="3"/>
       <c r="M1736" s="3"/>
       <c r="N1736" s="3"/>
+    </row>
+    <row r="1737" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1737" s="3" t="s">
+        <v>4368</v>
+      </c>
+      <c r="B1737" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1737" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1737" s="3">
+        <v>5993408319</v>
+      </c>
+      <c r="E1737" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1737" s="3" t="s">
+        <v>1483</v>
+      </c>
+      <c r="G1737" s="3" t="s">
+        <v>4369</v>
+      </c>
+      <c r="H1737" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="I1737" s="3">
+        <v>65</v>
+      </c>
+      <c r="J1737" s="3">
+        <v>-5</v>
+      </c>
+      <c r="K1737" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1737" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1737" s="3" t="s">
+        <v>4370</v>
+      </c>
+      <c r="N1737" s="3" t="s">
+        <v>4371</v>
+      </c>
+    </row>
+    <row r="1738" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1738" s="3" t="s">
+        <v>4372</v>
+      </c>
+      <c r="B1738" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="C1738" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1738" s="3">
+        <v>5993861246</v>
+      </c>
+      <c r="E1738" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1738" s="3" t="s">
+        <v>3431</v>
+      </c>
+      <c r="G1738" s="3" t="s">
+        <v>4373</v>
+      </c>
+      <c r="H1738" s="3" t="s">
+        <v>853</v>
+      </c>
+      <c r="I1738" s="3">
+        <v>15</v>
+      </c>
+      <c r="J1738" s="3"/>
+      <c r="K1738" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1738" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1738" s="3" t="s">
+        <v>4374</v>
+      </c>
+      <c r="N1738" s="3"/>
+    </row>
+    <row r="1739" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1739" s="3" t="s">
+        <v>4375</v>
+      </c>
+      <c r="B1739" s="3"/>
+      <c r="C1739" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1739" s="3">
+        <v>5993908948</v>
+      </c>
+      <c r="E1739" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1739" s="3" t="s">
+        <v>4182</v>
+      </c>
+      <c r="G1739" s="3" t="s">
+        <v>4376</v>
+      </c>
+      <c r="H1739" s="3"/>
+      <c r="I1739" s="3">
+        <v>51</v>
+      </c>
+      <c r="J1739" s="3">
+        <v>45</v>
+      </c>
+      <c r="K1739" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1739" s="3"/>
+      <c r="M1739" s="3"/>
+      <c r="N1739" s="3"/>
+    </row>
+    <row r="1740" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1740" s="3" t="s">
+        <v>4377</v>
+      </c>
+      <c r="B1740" s="3"/>
+      <c r="C1740" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1740" s="3">
+        <v>5994551829</v>
+      </c>
+      <c r="E1740" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1740" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1740" s="3" t="s">
+        <v>4378</v>
+      </c>
+      <c r="H1740" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="I1740" s="3">
+        <v>8</v>
+      </c>
+      <c r="J1740" s="3"/>
+      <c r="K1740" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1740" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1740" s="3" t="s">
+        <v>4379</v>
+      </c>
+      <c r="N1740" s="3"/>
+    </row>
+    <row r="1741" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1741" s="3" t="s">
+        <v>4380</v>
+      </c>
+      <c r="B1741" s="3"/>
+      <c r="C1741" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1741" s="3">
+        <v>5994912239</v>
+      </c>
+      <c r="E1741" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1741" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1741" s="3" t="s">
+        <v>4381</v>
+      </c>
+      <c r="H1741" s="3"/>
+      <c r="I1741" s="3">
+        <v>36</v>
+      </c>
+      <c r="J1741" s="3"/>
+      <c r="K1741" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1741" s="3"/>
+      <c r="M1741" s="3"/>
+      <c r="N1741" s="3"/>
+    </row>
+    <row r="1742" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1742" s="3" t="s">
+        <v>4382</v>
+      </c>
+      <c r="B1742" s="3"/>
+      <c r="C1742" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1742" s="3">
+        <v>5994976635</v>
+      </c>
+      <c r="E1742" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1742" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G1742" s="3" t="s">
+        <v>4383</v>
+      </c>
+      <c r="H1742" s="3"/>
+      <c r="I1742" s="3">
+        <v>42</v>
+      </c>
+      <c r="J1742" s="3"/>
+      <c r="K1742" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1742" s="3"/>
+      <c r="M1742" s="3"/>
+      <c r="N1742" s="3"/>
+    </row>
+    <row r="1743" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1743" s="3" t="s">
+        <v>4384</v>
+      </c>
+      <c r="B1743" s="3"/>
+      <c r="C1743" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1743" s="3">
+        <v>5995431874</v>
+      </c>
+      <c r="E1743" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F1743" s="3" t="s">
+        <v>4385</v>
+      </c>
+      <c r="G1743" s="3" t="s">
+        <v>4386</v>
+      </c>
+      <c r="H1743" s="3"/>
+      <c r="I1743" s="3">
+        <v>36</v>
+      </c>
+      <c r="J1743" s="3"/>
+      <c r="K1743" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1743" s="3"/>
+      <c r="M1743" s="3"/>
+      <c r="N1743" s="3"/>
+    </row>
+    <row r="1744" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1744" s="3" t="s">
+        <v>4387</v>
+      </c>
+      <c r="B1744" s="3"/>
+      <c r="C1744" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1744" s="3">
+        <v>5995522004</v>
+      </c>
+      <c r="E1744" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1744" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="G1744" s="3" t="s">
+        <v>4388</v>
+      </c>
+      <c r="H1744" s="3"/>
+      <c r="I1744" s="3">
+        <v>71</v>
+      </c>
+      <c r="J1744" s="3"/>
+      <c r="K1744" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1744" s="3"/>
+      <c r="M1744" s="3"/>
+      <c r="N1744" s="3"/>
+    </row>
+    <row r="1745" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1745" s="3" t="s">
+        <v>4389</v>
+      </c>
+      <c r="B1745" s="3"/>
+      <c r="C1745" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1745" s="3">
+        <v>5995893171</v>
+      </c>
+      <c r="E1745" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1745" s="3" t="s">
+        <v>4390</v>
+      </c>
+      <c r="G1745" s="3" t="s">
+        <v>4391</v>
+      </c>
+      <c r="H1745" s="3"/>
+      <c r="I1745" s="3"/>
+      <c r="J1745" s="3"/>
+      <c r="K1745" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1745" s="3"/>
+      <c r="M1745" s="3"/>
+      <c r="N1745" s="3"/>
+    </row>
+    <row r="1746" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1746" s="3" t="s">
+        <v>4392</v>
+      </c>
+      <c r="B1746" s="3"/>
+      <c r="C1746" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1746" s="3">
+        <v>5996022685</v>
+      </c>
+      <c r="E1746" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1746" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G1746" s="3" t="s">
+        <v>4393</v>
+      </c>
+      <c r="H1746" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="I1746" s="3">
+        <v>8</v>
+      </c>
+      <c r="J1746" s="3"/>
+      <c r="K1746" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1746" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1746" s="3" t="s">
+        <v>4394</v>
+      </c>
+      <c r="N1746" s="3"/>
+    </row>
+    <row r="1747" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1747" s="3" t="s">
+        <v>4395</v>
+      </c>
+      <c r="B1747" s="3"/>
+      <c r="C1747" s="3">
+        <v>2</v>
+      </c>
+      <c r="D1747" s="3">
+        <v>5996920759</v>
+      </c>
+      <c r="E1747" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F1747" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="G1747" s="3" t="s">
+        <v>4396</v>
+      </c>
+      <c r="H1747" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="I1747" s="3">
+        <v>74</v>
+      </c>
+      <c r="J1747" s="3">
+        <v>70</v>
+      </c>
+      <c r="K1747" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1747" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1747" s="3" t="s">
+        <v>4397</v>
+      </c>
+      <c r="N1747" s="3"/>
+    </row>
+    <row r="1748" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1748" s="3" t="s">
+        <v>4398</v>
+      </c>
+      <c r="B1748" s="3"/>
+      <c r="C1748" s="3">
+        <v>2</v>
+      </c>
+      <c r="D1748" s="3">
+        <v>5997423665</v>
+      </c>
+      <c r="E1748" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1748" s="3" t="s">
+        <v>4399</v>
+      </c>
+      <c r="G1748" s="3" t="s">
+        <v>4400</v>
+      </c>
+      <c r="H1748" s="3"/>
+      <c r="I1748" s="3">
+        <v>10</v>
+      </c>
+      <c r="J1748" s="3"/>
+      <c r="K1748" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1748" s="3"/>
+      <c r="M1748" s="3"/>
+      <c r="N1748" s="3"/>
+    </row>
+    <row r="1749" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1749" s="3" t="s">
+        <v>4401</v>
+      </c>
+      <c r="B1749" s="3"/>
+      <c r="C1749" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1749" s="3">
+        <v>5997695451</v>
+      </c>
+      <c r="E1749" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1749" s="3" t="s">
+        <v>4402</v>
+      </c>
+      <c r="G1749" s="3" t="s">
+        <v>4403</v>
+      </c>
+      <c r="H1749" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="I1749" s="3">
+        <v>67</v>
+      </c>
+      <c r="J1749" s="3"/>
+      <c r="K1749" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1749" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1749" s="3" t="s">
+        <v>4404</v>
+      </c>
+      <c r="N1749" s="3"/>
+    </row>
+    <row r="1750" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1750" s="3" t="s">
+        <v>4405</v>
+      </c>
+      <c r="B1750" s="3"/>
+      <c r="C1750" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1750" s="3">
+        <v>5998088844</v>
+      </c>
+      <c r="E1750" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1750" s="3" t="s">
+        <v>4406</v>
+      </c>
+      <c r="G1750" s="3" t="s">
+        <v>4407</v>
+      </c>
+      <c r="H1750" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="I1750" s="3">
+        <v>11</v>
+      </c>
+      <c r="J1750" s="3"/>
+      <c r="K1750" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1750" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1750" s="3" t="s">
+        <v>4408</v>
+      </c>
+      <c r="N1750" s="3"/>
+    </row>
+    <row r="1751" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1751" s="3" t="s">
+        <v>4409</v>
+      </c>
+      <c r="B1751" s="3"/>
+      <c r="C1751" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1751" s="3">
+        <v>5998532627</v>
+      </c>
+      <c r="E1751" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1751" s="3" t="s">
+        <v>2161</v>
+      </c>
+      <c r="G1751" s="3" t="s">
+        <v>4410</v>
+      </c>
+      <c r="H1751" s="3"/>
+      <c r="I1751" s="3">
+        <v>68</v>
+      </c>
+      <c r="J1751" s="3"/>
+      <c r="K1751" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1751" s="3"/>
+      <c r="M1751" s="3"/>
+      <c r="N1751" s="3"/>
+    </row>
+    <row r="1752" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1752" s="3" t="s">
+        <v>4411</v>
+      </c>
+      <c r="B1752" s="3"/>
+      <c r="C1752" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1752" s="3">
+        <v>5999156571</v>
+      </c>
+      <c r="E1752" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1752" s="3" t="s">
+        <v>946</v>
+      </c>
+      <c r="G1752" s="3" t="s">
+        <v>4412</v>
+      </c>
+      <c r="H1752" s="3"/>
+      <c r="I1752" s="3">
+        <v>67</v>
+      </c>
+      <c r="J1752" s="3">
+        <v>60</v>
+      </c>
+      <c r="K1752" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1752" s="3"/>
+      <c r="M1752" s="3"/>
+      <c r="N1752" s="3"/>
+    </row>
+    <row r="1753" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1753" s="3" t="s">
+        <v>4413</v>
+      </c>
+      <c r="B1753" s="3"/>
+      <c r="C1753" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1753" s="3">
+        <v>5999177768</v>
+      </c>
+      <c r="E1753" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1753" s="3" t="s">
+        <v>1968</v>
+      </c>
+      <c r="G1753" s="3" t="s">
+        <v>4414</v>
+      </c>
+      <c r="H1753" s="3"/>
+      <c r="I1753" s="3">
+        <v>60</v>
+      </c>
+      <c r="J1753" s="3">
+        <v>50</v>
+      </c>
+      <c r="K1753" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1753" s="3"/>
+      <c r="M1753" s="3"/>
+      <c r="N1753" s="3"/>
+    </row>
+    <row r="1754" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1754" s="3" t="s">
+        <v>4415</v>
+      </c>
+      <c r="B1754" s="3"/>
+      <c r="C1754" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1754" s="3">
+        <v>6000878480</v>
+      </c>
+      <c r="E1754" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1754" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="G1754" s="3" t="s">
+        <v>4416</v>
+      </c>
+      <c r="H1754" s="3"/>
+      <c r="I1754" s="3">
+        <v>61</v>
+      </c>
+      <c r="J1754" s="3">
+        <v>50</v>
+      </c>
+      <c r="K1754" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1754" s="3"/>
+      <c r="M1754" s="3"/>
+      <c r="N1754" s="3"/>
+    </row>
+    <row r="1755" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1755" s="3" t="s">
+        <v>4417</v>
+      </c>
+      <c r="B1755" s="3"/>
+      <c r="C1755" s="3">
+        <v>2</v>
+      </c>
+      <c r="D1755" s="3">
+        <v>6001325514</v>
+      </c>
+      <c r="E1755" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1755" s="3" t="s">
+        <v>4418</v>
+      </c>
+      <c r="G1755" s="3" t="s">
+        <v>4419</v>
+      </c>
+      <c r="H1755" s="3"/>
+      <c r="I1755" s="3">
+        <v>58</v>
+      </c>
+      <c r="J1755" s="3">
+        <v>45</v>
+      </c>
+      <c r="K1755" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1755" s="3"/>
+      <c r="M1755" s="3"/>
+      <c r="N1755" s="3"/>
+    </row>
+    <row r="1756" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1756" s="3" t="s">
+        <v>4420</v>
+      </c>
+      <c r="B1756" s="3"/>
+      <c r="C1756" s="3">
+        <v>26</v>
+      </c>
+      <c r="D1756" s="3">
+        <v>6001885083</v>
+      </c>
+      <c r="E1756" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1756" s="3" t="s">
+        <v>2061</v>
+      </c>
+      <c r="G1756" s="3" t="s">
+        <v>4421</v>
+      </c>
+      <c r="H1756" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="I1756" s="3">
+        <v>60</v>
+      </c>
+      <c r="J1756" s="3"/>
+      <c r="K1756" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1756" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1756" s="3" t="s">
+        <v>4422</v>
+      </c>
+      <c r="N1756" s="3"/>
+    </row>
+    <row r="1757" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1757" s="3" t="s">
+        <v>4423</v>
+      </c>
+      <c r="B1757" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="C1757" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1757" s="3">
+        <v>6002528364</v>
+      </c>
+      <c r="E1757" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1757" s="3" t="s">
+        <v>4424</v>
+      </c>
+      <c r="G1757" s="3" t="s">
+        <v>4425</v>
+      </c>
+      <c r="H1757" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="I1757" s="3">
+        <v>65</v>
+      </c>
+      <c r="J1757" s="3"/>
+      <c r="K1757" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1757" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1757" s="3" t="s">
+        <v>4426</v>
+      </c>
+      <c r="N1757" s="3" t="s">
+        <v>4427</v>
+      </c>
+    </row>
+    <row r="1758" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1758" s="3" t="s">
+        <v>4428</v>
+      </c>
+      <c r="B1758" s="3"/>
+      <c r="C1758" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1758" s="3">
+        <v>6003880110</v>
+      </c>
+      <c r="E1758" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1758" s="3" t="s">
+        <v>1075</v>
+      </c>
+      <c r="G1758" s="3" t="s">
+        <v>4429</v>
+      </c>
+      <c r="H1758" s="3"/>
+      <c r="I1758" s="3">
+        <v>27</v>
+      </c>
+      <c r="J1758" s="3"/>
+      <c r="K1758" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1758" s="3"/>
+      <c r="M1758" s="3"/>
+      <c r="N1758" s="3"/>
+    </row>
+    <row r="1759" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1759" s="3" t="s">
+        <v>4430</v>
+      </c>
+      <c r="B1759" s="3"/>
+      <c r="C1759" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1759" s="3">
+        <v>6003918664</v>
+      </c>
+      <c r="E1759" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1759" s="3" t="s">
+        <v>4431</v>
+      </c>
+      <c r="G1759" s="3" t="s">
+        <v>4432</v>
+      </c>
+      <c r="H1759" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="I1759" s="3">
+        <v>71</v>
+      </c>
+      <c r="J1759" s="3"/>
+      <c r="K1759" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1759" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1759" s="3" t="s">
+        <v>4427</v>
+      </c>
+      <c r="N1759" s="3"/>
+    </row>
+    <row r="1760" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1760" s="3" t="s">
+        <v>4433</v>
+      </c>
+      <c r="B1760" s="3"/>
+      <c r="C1760" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1760" s="3">
+        <v>6004011095</v>
+      </c>
+      <c r="E1760" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1760" s="3" t="s">
+        <v>4434</v>
+      </c>
+      <c r="G1760" s="3" t="s">
+        <v>4435</v>
+      </c>
+      <c r="H1760" s="3"/>
+      <c r="I1760" s="3">
+        <v>69</v>
+      </c>
+      <c r="J1760" s="3">
+        <v>60</v>
+      </c>
+      <c r="K1760" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1760" s="3"/>
+      <c r="M1760" s="3"/>
+      <c r="N1760" s="3"/>
+    </row>
+    <row r="1761" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1761" s="3" t="s">
+        <v>4436</v>
+      </c>
+      <c r="B1761" s="3"/>
+      <c r="C1761" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1761" s="3">
+        <v>6004136799</v>
+      </c>
+      <c r="E1761" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1761" s="3" t="s">
+        <v>4437</v>
+      </c>
+      <c r="G1761" s="3" t="s">
+        <v>4438</v>
+      </c>
+      <c r="H1761" s="3"/>
+      <c r="I1761" s="3">
+        <v>66</v>
+      </c>
+      <c r="J1761" s="3">
+        <v>60</v>
+      </c>
+      <c r="K1761" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1761" s="3"/>
+      <c r="M1761" s="3"/>
+      <c r="N1761" s="3"/>
+    </row>
+    <row r="1762" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1762" s="3" t="s">
+        <v>4439</v>
+      </c>
+      <c r="B1762" s="3"/>
+      <c r="C1762" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1762" s="3">
+        <v>6004146042</v>
+      </c>
+      <c r="E1762" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1762" s="3" t="s">
+        <v>2620</v>
+      </c>
+      <c r="G1762" s="3" t="s">
+        <v>4440</v>
+      </c>
+      <c r="H1762" s="3"/>
+      <c r="I1762" s="3">
+        <v>62</v>
+      </c>
+      <c r="J1762" s="3">
+        <v>55</v>
+      </c>
+      <c r="K1762" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1762" s="3"/>
+      <c r="M1762" s="3"/>
+      <c r="N1762" s="3"/>
+    </row>
+    <row r="1763" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1763" s="3" t="s">
+        <v>4441</v>
+      </c>
+      <c r="B1763" s="3"/>
+      <c r="C1763" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1763" s="3">
+        <v>6004695537</v>
+      </c>
+      <c r="E1763" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1763" s="3" t="s">
+        <v>4442</v>
+      </c>
+      <c r="G1763" s="3" t="s">
+        <v>4443</v>
+      </c>
+      <c r="H1763" s="3"/>
+      <c r="I1763" s="3">
+        <v>76</v>
+      </c>
+      <c r="J1763" s="3"/>
+      <c r="K1763" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1763" s="3"/>
+      <c r="M1763" s="3"/>
+      <c r="N1763" s="3"/>
+    </row>
+    <row r="1764" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1764" s="3" t="s">
+        <v>4444</v>
+      </c>
+      <c r="B1764" s="3"/>
+      <c r="C1764" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1764" s="3">
+        <v>6005812755</v>
+      </c>
+      <c r="E1764" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1764" s="3" t="s">
+        <v>4445</v>
+      </c>
+      <c r="G1764" s="3" t="s">
+        <v>4446</v>
+      </c>
+      <c r="H1764" s="3"/>
+      <c r="I1764" s="3">
+        <v>57</v>
+      </c>
+      <c r="J1764" s="3">
+        <v>50</v>
+      </c>
+      <c r="K1764" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1764" s="3"/>
+      <c r="M1764" s="3"/>
+      <c r="N1764" s="3"/>
+    </row>
+    <row r="1765" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1765" s="3" t="s">
+        <v>4447</v>
+      </c>
+      <c r="B1765" s="3"/>
+      <c r="C1765" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1765" s="3">
+        <v>6007562741</v>
+      </c>
+      <c r="E1765" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1765" s="3" t="s">
+        <v>3273</v>
+      </c>
+      <c r="G1765" s="3" t="s">
+        <v>4448</v>
+      </c>
+      <c r="H1765" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="I1765" s="3">
+        <v>33</v>
+      </c>
+      <c r="J1765" s="3"/>
+      <c r="K1765" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1765" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1765" s="3" t="s">
+        <v>4449</v>
+      </c>
+      <c r="N1765" s="3"/>
+    </row>
+    <row r="1766" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1766" s="3" t="s">
+        <v>4450</v>
+      </c>
+      <c r="B1766" s="3"/>
+      <c r="C1766" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1766" s="3">
+        <v>6007590533</v>
+      </c>
+      <c r="E1766" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1766" s="3" t="s">
+        <v>856</v>
+      </c>
+      <c r="G1766" s="3" t="s">
+        <v>4451</v>
+      </c>
+      <c r="H1766" s="3"/>
+      <c r="I1766" s="3">
+        <v>80</v>
+      </c>
+      <c r="J1766" s="3">
+        <v>70</v>
+      </c>
+      <c r="K1766" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1766" s="3"/>
+      <c r="M1766" s="3"/>
+      <c r="N1766" s="3"/>
+    </row>
+    <row r="1767" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1767" s="3" t="s">
+        <v>4452</v>
+      </c>
+      <c r="B1767" s="3"/>
+      <c r="C1767" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1767" s="3">
+        <v>6007616594</v>
+      </c>
+      <c r="E1767" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="F1767" s="3" t="s">
+        <v>1143</v>
+      </c>
+      <c r="G1767" s="3" t="s">
+        <v>4453</v>
+      </c>
+      <c r="H1767" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="I1767" s="3"/>
+      <c r="J1767" s="3"/>
+      <c r="K1767" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1767" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1767" s="3" t="s">
+        <v>4449</v>
+      </c>
+      <c r="N1767" s="3"/>
+    </row>
+    <row r="1768" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1768" s="3" t="s">
+        <v>4454</v>
+      </c>
+      <c r="B1768" s="3"/>
+      <c r="C1768" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1768" s="3">
+        <v>6008078539</v>
+      </c>
+      <c r="E1768" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1768" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="G1768" s="3" t="s">
+        <v>4455</v>
+      </c>
+      <c r="H1768" s="3"/>
+      <c r="I1768" s="3">
+        <v>16</v>
+      </c>
+      <c r="J1768" s="3"/>
+      <c r="K1768" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1768" s="3"/>
+      <c r="M1768" s="3"/>
+      <c r="N1768" s="3"/>
+    </row>
+    <row r="1769" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1769" s="3" t="s">
+        <v>4456</v>
+      </c>
+      <c r="B1769" s="3"/>
+      <c r="C1769" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1769" s="3">
+        <v>6012425169</v>
+      </c>
+      <c r="E1769" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1769" s="3" t="s">
+        <v>2149</v>
+      </c>
+      <c r="G1769" s="3" t="s">
+        <v>4457</v>
+      </c>
+      <c r="H1769" s="3"/>
+      <c r="I1769" s="3">
+        <v>61</v>
+      </c>
+      <c r="J1769" s="3"/>
+      <c r="K1769" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1769" s="3"/>
+      <c r="M1769" s="3"/>
+      <c r="N1769" s="3"/>
+    </row>
+    <row r="1770" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1770" s="3" t="s">
+        <v>4458</v>
+      </c>
+      <c r="B1770" s="3"/>
+      <c r="C1770" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1770" s="3">
+        <v>6014015211</v>
+      </c>
+      <c r="E1770" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1770" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="G1770" s="3" t="s">
+        <v>4459</v>
+      </c>
+      <c r="H1770" s="3"/>
+      <c r="I1770" s="3">
+        <v>37</v>
+      </c>
+      <c r="J1770" s="3"/>
+      <c r="K1770" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1770" s="3"/>
+      <c r="M1770" s="3"/>
+      <c r="N1770" s="3"/>
+    </row>
+    <row r="1771" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1771" s="3" t="s">
+        <v>4460</v>
+      </c>
+      <c r="B1771" s="3"/>
+      <c r="C1771" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1771" s="3">
+        <v>6014166286</v>
+      </c>
+      <c r="E1771" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="F1771" s="3" t="s">
+        <v>1148</v>
+      </c>
+      <c r="G1771" s="3" t="s">
+        <v>4461</v>
+      </c>
+      <c r="H1771" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="I1771" s="3">
+        <v>11</v>
+      </c>
+      <c r="J1771" s="3"/>
+      <c r="K1771" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1771" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1771" s="3" t="s">
+        <v>4462</v>
+      </c>
+      <c r="N1771" s="3"/>
+    </row>
+    <row r="1772" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1772" s="3" t="s">
+        <v>4463</v>
+      </c>
+      <c r="B1772" s="3"/>
+      <c r="C1772" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1772" s="3">
+        <v>6014170348</v>
+      </c>
+      <c r="E1772" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F1772" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="G1772" s="3" t="s">
+        <v>4464</v>
+      </c>
+      <c r="H1772" s="3"/>
+      <c r="I1772" s="3">
+        <v>37</v>
+      </c>
+      <c r="J1772" s="3"/>
+      <c r="K1772" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1772" s="3"/>
+      <c r="M1772" s="3"/>
+      <c r="N1772" s="3"/>
+    </row>
+    <row r="1773" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1773" s="3" t="s">
+        <v>4465</v>
+      </c>
+      <c r="B1773" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="C1773" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1773" s="3">
+        <v>6015254777</v>
+      </c>
+      <c r="E1773" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="F1773" s="3" t="s">
+        <v>1948</v>
+      </c>
+      <c r="G1773" s="3" t="s">
+        <v>4466</v>
+      </c>
+      <c r="H1773" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="I1773" s="3">
+        <v>50</v>
+      </c>
+      <c r="J1773" s="3"/>
+      <c r="K1773" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1773" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1773" s="3" t="s">
+        <v>4467</v>
+      </c>
+      <c r="N1773" s="3"/>
+    </row>
+    <row r="1774" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1774" s="3" t="s">
+        <v>4468</v>
+      </c>
+      <c r="B1774" s="3"/>
+      <c r="C1774" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1774" s="3">
+        <v>6015678766</v>
+      </c>
+      <c r="E1774" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1774" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G1774" s="3" t="s">
+        <v>4469</v>
+      </c>
+      <c r="H1774" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="I1774" s="3">
+        <v>7</v>
+      </c>
+      <c r="J1774" s="3"/>
+      <c r="K1774" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1774" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1774" s="3" t="s">
+        <v>4470</v>
+      </c>
+      <c r="N1774" s="3"/>
+    </row>
+    <row r="1775" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1775" s="3" t="s">
+        <v>4471</v>
+      </c>
+      <c r="B1775" s="3"/>
+      <c r="C1775" s="3">
+        <v>26</v>
+      </c>
+      <c r="D1775" s="3">
+        <v>6018308358</v>
+      </c>
+      <c r="E1775" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F1775" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="G1775" s="3" t="s">
+        <v>4472</v>
+      </c>
+      <c r="H1775" s="3"/>
+      <c r="I1775" s="3"/>
+      <c r="J1775" s="3"/>
+      <c r="K1775" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1775" s="3"/>
+      <c r="M1775" s="3"/>
+      <c r="N1775" s="3"/>
+    </row>
+    <row r="1776" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1776" s="3" t="s">
+        <v>4473</v>
+      </c>
+      <c r="B1776" s="3"/>
+      <c r="C1776" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1776" s="3">
+        <v>6018621293</v>
+      </c>
+      <c r="E1776" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1776" s="3" t="s">
+        <v>914</v>
+      </c>
+      <c r="G1776" s="3" t="s">
+        <v>4474</v>
+      </c>
+      <c r="H1776" s="3"/>
+      <c r="I1776" s="3"/>
+      <c r="J1776" s="3"/>
+      <c r="K1776" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1776" s="3"/>
+      <c r="M1776" s="3"/>
+      <c r="N1776" s="3"/>
+    </row>
+    <row r="1777" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1777" s="3" t="s">
+        <v>4475</v>
+      </c>
+      <c r="B1777" s="3"/>
+      <c r="C1777" s="3">
+        <v>26</v>
+      </c>
+      <c r="D1777" s="3">
+        <v>6018681485</v>
+      </c>
+      <c r="E1777" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1777" s="3" t="s">
+        <v>1818</v>
+      </c>
+      <c r="G1777" s="3" t="s">
+        <v>4476</v>
+      </c>
+      <c r="H1777" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="I1777" s="3"/>
+      <c r="J1777" s="3"/>
+      <c r="K1777" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1777" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1777" s="3" t="s">
+        <v>4470</v>
+      </c>
+      <c r="N1777" s="3"/>
+    </row>
+    <row r="1778" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1778" s="3" t="s">
+        <v>4477</v>
+      </c>
+      <c r="B1778" s="3"/>
+      <c r="C1778" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1778" s="3">
+        <v>6019207726</v>
+      </c>
+      <c r="E1778" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1778" s="3" t="s">
+        <v>4478</v>
+      </c>
+      <c r="G1778" s="3" t="s">
+        <v>4479</v>
+      </c>
+      <c r="H1778" s="3"/>
+      <c r="I1778" s="3"/>
+      <c r="J1778" s="3"/>
+      <c r="K1778" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1778" s="3"/>
+      <c r="M1778" s="3"/>
+      <c r="N1778" s="3"/>
+    </row>
+    <row r="1779" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1779" s="3" t="s">
+        <v>4480</v>
+      </c>
+      <c r="B1779" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1779" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1779" s="3">
+        <v>6019257431</v>
+      </c>
+      <c r="E1779" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1779" s="3" t="s">
+        <v>1472</v>
+      </c>
+      <c r="G1779" s="3" t="s">
+        <v>4481</v>
+      </c>
+      <c r="H1779" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="I1779" s="3"/>
+      <c r="J1779" s="3"/>
+      <c r="K1779" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1779" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1779" s="3" t="s">
+        <v>4482</v>
+      </c>
+      <c r="N1779" s="3" t="s">
+        <v>4483</v>
+      </c>
+    </row>
+    <row r="1780" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1780" s="3" t="s">
+        <v>4484</v>
+      </c>
+      <c r="B1780" s="3"/>
+      <c r="C1780" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1780" s="3">
+        <v>6019716450</v>
+      </c>
+      <c r="E1780" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1780" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="G1780" s="3" t="s">
+        <v>4485</v>
+      </c>
+      <c r="H1780" s="3"/>
+      <c r="I1780" s="3"/>
+      <c r="J1780" s="3"/>
+      <c r="K1780" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1780" s="3"/>
+      <c r="M1780" s="3"/>
+      <c r="N1780" s="3"/>
+    </row>
+    <row r="1781" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1781" s="3" t="s">
+        <v>4486</v>
+      </c>
+      <c r="B1781" s="3"/>
+      <c r="C1781" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1781" s="3">
+        <v>6022274866</v>
+      </c>
+      <c r="E1781" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1781" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1781" s="3" t="s">
+        <v>4487</v>
+      </c>
+      <c r="H1781" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="I1781" s="3">
+        <v>9</v>
+      </c>
+      <c r="J1781" s="3"/>
+      <c r="K1781" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="L1781" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="M1781" s="3" t="s">
+        <v>4488</v>
+      </c>
+      <c r="N1781" s="3"/>
+    </row>
+    <row r="1782" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1782" s="3" t="s">
+        <v>4489</v>
+      </c>
+      <c r="B1782" s="3"/>
+      <c r="C1782" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1782" s="3">
+        <v>6022446607</v>
+      </c>
+      <c r="E1782" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1782" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="G1782" s="3" t="s">
+        <v>4490</v>
+      </c>
+      <c r="H1782" s="3"/>
+      <c r="I1782" s="3">
+        <v>14</v>
+      </c>
+      <c r="J1782" s="3"/>
+      <c r="K1782" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1782" s="3"/>
+      <c r="M1782" s="3"/>
+      <c r="N1782" s="3"/>
+    </row>
+    <row r="1783" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1783" s="3" t="s">
+        <v>4491</v>
+      </c>
+      <c r="B1783" s="3"/>
+      <c r="C1783" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1783" s="3">
+        <v>6022519055</v>
+      </c>
+      <c r="E1783" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1783" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G1783" s="3" t="s">
+        <v>4492</v>
+      </c>
+      <c r="H1783" s="3"/>
+      <c r="I1783" s="3">
+        <v>56</v>
+      </c>
+      <c r="J1783" s="3">
+        <v>50</v>
+      </c>
+      <c r="K1783" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1783" s="3"/>
+      <c r="M1783" s="3"/>
+      <c r="N1783" s="3"/>
+    </row>
+    <row r="1784" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1784" s="3" t="s">
+        <v>4493</v>
+      </c>
+      <c r="B1784" s="3"/>
+      <c r="C1784" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1784" s="3">
+        <v>6024059951</v>
+      </c>
+      <c r="E1784" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1784" s="3" t="s">
+        <v>528</v>
+      </c>
+      <c r="G1784" s="3" t="s">
+        <v>4494</v>
+      </c>
+      <c r="H1784" s="3"/>
+      <c r="I1784" s="3">
+        <v>74</v>
+      </c>
+      <c r="J1784" s="3">
+        <v>70</v>
+      </c>
+      <c r="K1784" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1784" s="3"/>
+      <c r="M1784" s="3"/>
+      <c r="N1784" s="3"/>
+    </row>
+    <row r="1785" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1785" s="3" t="s">
+        <v>4493</v>
+      </c>
+      <c r="B1785" s="3"/>
+      <c r="C1785" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1785" s="3">
+        <v>6024060291</v>
+      </c>
+      <c r="E1785" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1785" s="3" t="s">
+        <v>4495</v>
+      </c>
+      <c r="G1785" s="3" t="s">
+        <v>4496</v>
+      </c>
+      <c r="H1785" s="3"/>
+      <c r="I1785" s="3">
+        <v>37</v>
+      </c>
+      <c r="J1785" s="3"/>
+      <c r="K1785" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1785" s="3"/>
+      <c r="M1785" s="3"/>
+      <c r="N1785" s="3"/>
+    </row>
+    <row r="1786" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1786" s="3" t="s">
+        <v>4497</v>
+      </c>
+      <c r="B1786" s="3"/>
+      <c r="C1786" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1786" s="3">
+        <v>6024101955</v>
+      </c>
+      <c r="E1786" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1786" s="3" t="s">
+        <v>801</v>
+      </c>
+      <c r="G1786" s="3" t="s">
+        <v>4498</v>
+      </c>
+      <c r="H1786" s="3"/>
+      <c r="I1786" s="3">
+        <v>71</v>
+      </c>
+      <c r="J1786" s="3"/>
+      <c r="K1786" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1786" s="3"/>
+      <c r="M1786" s="3"/>
+      <c r="N1786" s="3"/>
+    </row>
+    <row r="1787" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1787" s="3" t="s">
+        <v>4499</v>
+      </c>
+      <c r="B1787" s="3"/>
+      <c r="C1787" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1787" s="3">
+        <v>6024280818</v>
+      </c>
+      <c r="E1787" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1787" s="3" t="s">
+        <v>4500</v>
+      </c>
+      <c r="G1787" s="3" t="s">
+        <v>4501</v>
+      </c>
+      <c r="H1787" s="3"/>
+      <c r="I1787" s="3">
+        <v>76</v>
+      </c>
+      <c r="J1787" s="3">
+        <v>70</v>
+      </c>
+      <c r="K1787" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1787" s="3"/>
+      <c r="M1787" s="3"/>
+      <c r="N1787" s="3"/>
+    </row>
+    <row r="1788" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1788" s="3" t="s">
+        <v>4502</v>
+      </c>
+      <c r="B1788" s="3"/>
+      <c r="C1788" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1788" s="3">
+        <v>6024425113</v>
+      </c>
+      <c r="E1788" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1788" s="3" t="s">
+        <v>4503</v>
+      </c>
+      <c r="G1788" s="3" t="s">
+        <v>4504</v>
+      </c>
+      <c r="H1788" s="3"/>
+      <c r="I1788" s="3">
+        <v>2</v>
+      </c>
+      <c r="J1788" s="3"/>
+      <c r="K1788" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1788" s="3"/>
+      <c r="M1788" s="3"/>
+      <c r="N1788" s="3"/>
+    </row>
+    <row r="1789" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1789" s="3" t="s">
+        <v>4505</v>
+      </c>
+      <c r="B1789" s="3"/>
+      <c r="C1789" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1789" s="3">
+        <v>6024589225</v>
+      </c>
+      <c r="E1789" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1789" s="3" t="s">
+        <v>4506</v>
+      </c>
+      <c r="G1789" s="3" t="s">
+        <v>4507</v>
+      </c>
+      <c r="H1789" s="3"/>
+      <c r="I1789" s="3">
+        <v>68</v>
+      </c>
+      <c r="J1789" s="3"/>
+      <c r="K1789" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1789" s="3"/>
+      <c r="M1789" s="3"/>
+      <c r="N1789" s="3"/>
+    </row>
+    <row r="1790" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1790" s="3" t="s">
+        <v>4508</v>
+      </c>
+      <c r="B1790" s="3"/>
+      <c r="C1790" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1790" s="3">
+        <v>6024791252</v>
+      </c>
+      <c r="E1790" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="F1790" s="3" t="s">
+        <v>1090</v>
+      </c>
+      <c r="G1790" s="3" t="s">
+        <v>4509</v>
+      </c>
+      <c r="H1790" s="3"/>
+      <c r="I1790" s="3">
+        <v>67</v>
+      </c>
+      <c r="J1790" s="3"/>
+      <c r="K1790" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1790" s="3"/>
+      <c r="M1790" s="3"/>
+      <c r="N1790" s="3"/>
+    </row>
+    <row r="1791" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1791" s="3" t="s">
+        <v>4510</v>
+      </c>
+      <c r="B1791" s="3"/>
+      <c r="C1791" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1791" s="3">
+        <v>6024836205</v>
+      </c>
+      <c r="E1791" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="F1791" s="3" t="s">
+        <v>2375</v>
+      </c>
+      <c r="G1791" s="3" t="s">
+        <v>4511</v>
+      </c>
+      <c r="H1791" s="3"/>
+      <c r="I1791" s="3">
+        <v>75</v>
+      </c>
+      <c r="J1791" s="3"/>
+      <c r="K1791" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1791" s="3"/>
+      <c r="M1791" s="3"/>
+      <c r="N1791" s="3"/>
+    </row>
+    <row r="1792" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1792" s="3" t="s">
+        <v>4512</v>
+      </c>
+      <c r="B1792" s="3"/>
+      <c r="C1792" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1792" s="3">
+        <v>6024854593</v>
+      </c>
+      <c r="E1792" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1792" s="3" t="s">
+        <v>1148</v>
+      </c>
+      <c r="G1792" s="3" t="s">
+        <v>4513</v>
+      </c>
+      <c r="H1792" s="3"/>
+      <c r="I1792" s="3">
+        <v>76</v>
+      </c>
+      <c r="J1792" s="3"/>
+      <c r="K1792" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1792" s="3"/>
+      <c r="M1792" s="3"/>
+      <c r="N1792" s="3"/>
+    </row>
+    <row r="1793" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1793" s="3" t="s">
+        <v>4514</v>
+      </c>
+      <c r="B1793" s="3"/>
+      <c r="C1793" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1793" s="3">
+        <v>6024854598</v>
+      </c>
+      <c r="E1793" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1793" s="3" t="s">
+        <v>892</v>
+      </c>
+      <c r="G1793" s="3" t="s">
+        <v>4515</v>
+      </c>
+      <c r="H1793" s="3"/>
+      <c r="I1793" s="3">
+        <v>70</v>
+      </c>
+      <c r="J1793" s="3">
+        <v>70</v>
+      </c>
+      <c r="K1793" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1793" s="3"/>
+      <c r="M1793" s="3"/>
+      <c r="N1793" s="3"/>
+    </row>
+    <row r="1794" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1794" s="3" t="s">
+        <v>4516</v>
+      </c>
+      <c r="B1794" s="3"/>
+      <c r="C1794" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1794" s="3">
+        <v>6025434736</v>
+      </c>
+      <c r="E1794" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1794" s="3" t="s">
+        <v>4517</v>
+      </c>
+      <c r="G1794" s="3" t="s">
+        <v>4518</v>
+      </c>
+      <c r="H1794" s="3"/>
+      <c r="I1794" s="3"/>
+      <c r="J1794" s="3"/>
+      <c r="K1794" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1794" s="3"/>
+      <c r="M1794" s="3"/>
+      <c r="N1794" s="3"/>
+    </row>
+    <row r="1795" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1795" s="3" t="s">
+        <v>4519</v>
+      </c>
+      <c r="B1795" s="3"/>
+      <c r="C1795" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1795" s="3">
+        <v>6025787949</v>
+      </c>
+      <c r="E1795" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1795" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="G1795" s="3" t="s">
+        <v>4520</v>
+      </c>
+      <c r="H1795" s="3"/>
+      <c r="I1795" s="3">
+        <v>75</v>
+      </c>
+      <c r="J1795" s="3"/>
+      <c r="K1795" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1795" s="3"/>
+      <c r="M1795" s="3"/>
+      <c r="N1795" s="3"/>
+    </row>
+    <row r="1796" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1796" s="3" t="s">
+        <v>4521</v>
+      </c>
+      <c r="B1796" s="3"/>
+      <c r="C1796" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1796" s="3">
+        <v>6027673212</v>
+      </c>
+      <c r="E1796" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1796" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="G1796" s="3" t="s">
+        <v>4522</v>
+      </c>
+      <c r="H1796" s="3"/>
+      <c r="I1796" s="3">
+        <v>67</v>
+      </c>
+      <c r="J1796" s="3">
+        <v>60</v>
+      </c>
+      <c r="K1796" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1796" s="3"/>
+      <c r="M1796" s="3"/>
+      <c r="N1796" s="3"/>
+    </row>
+    <row r="1797" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1797" s="3" t="s">
+        <v>4523</v>
+      </c>
+      <c r="B1797" s="3"/>
+      <c r="C1797" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1797" s="3">
+        <v>6030149799</v>
+      </c>
+      <c r="E1797" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1797" s="3" t="s">
+        <v>4524</v>
+      </c>
+      <c r="G1797" s="3" t="s">
+        <v>4525</v>
+      </c>
+      <c r="H1797" s="3"/>
+      <c r="I1797" s="3">
+        <v>65</v>
+      </c>
+      <c r="J1797" s="3"/>
+      <c r="K1797" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1797" s="3"/>
+      <c r="M1797" s="3"/>
+      <c r="N1797" s="3"/>
+    </row>
+    <row r="1798" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1798" s="3" t="s">
+        <v>4526</v>
+      </c>
+      <c r="B1798" s="3"/>
+      <c r="C1798" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1798" s="3">
+        <v>6030231305</v>
+      </c>
+      <c r="E1798" s="3" t="s">
+        <v>624</v>
+      </c>
+      <c r="F1798" s="3" t="s">
+        <v>4527</v>
+      </c>
+      <c r="G1798" s="3" t="s">
+        <v>4528</v>
+      </c>
+      <c r="H1798" s="3"/>
+      <c r="I1798" s="3">
+        <v>10</v>
+      </c>
+      <c r="J1798" s="3"/>
+      <c r="K1798" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1798" s="3"/>
+      <c r="M1798" s="3"/>
+      <c r="N1798" s="3"/>
+    </row>
+    <row r="1799" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1799" s="3" t="s">
+        <v>4529</v>
+      </c>
+      <c r="B1799" s="3"/>
+      <c r="C1799" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1799" s="3">
+        <v>6030231315</v>
+      </c>
+      <c r="E1799" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1799" s="3" t="s">
+        <v>4530</v>
+      </c>
+      <c r="G1799" s="3" t="s">
+        <v>4531</v>
+      </c>
+      <c r="H1799" s="3"/>
+      <c r="I1799" s="3">
+        <v>25</v>
+      </c>
+      <c r="J1799" s="3"/>
+      <c r="K1799" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1799" s="3"/>
+      <c r="M1799" s="3"/>
+      <c r="N1799" s="3"/>
+    </row>
+    <row r="1800" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1800" s="3" t="s">
+        <v>4532</v>
+      </c>
+      <c r="B1800" s="3"/>
+      <c r="C1800" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1800" s="3">
+        <v>6030391762</v>
+      </c>
+      <c r="E1800" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1800" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="G1800" s="3" t="s">
+        <v>4533</v>
+      </c>
+      <c r="H1800" s="3"/>
+      <c r="I1800" s="3">
+        <v>69</v>
+      </c>
+      <c r="J1800" s="3"/>
+      <c r="K1800" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1800" s="3"/>
+      <c r="M1800" s="3"/>
+      <c r="N1800" s="3"/>
+    </row>
+    <row r="1801" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1801" s="3" t="s">
+        <v>4534</v>
+      </c>
+      <c r="B1801" s="3"/>
+      <c r="C1801" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1801" s="3">
+        <v>6032973603</v>
+      </c>
+      <c r="E1801" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1801" s="3" t="s">
+        <v>1668</v>
+      </c>
+      <c r="G1801" s="3" t="s">
+        <v>4535</v>
+      </c>
+      <c r="H1801" s="3"/>
+      <c r="I1801" s="3">
+        <v>4</v>
+      </c>
+      <c r="J1801" s="3"/>
+      <c r="K1801" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1801" s="3"/>
+      <c r="M1801" s="3"/>
+      <c r="N1801" s="3"/>
+    </row>
+    <row r="1802" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1802" s="3" t="s">
+        <v>4536</v>
+      </c>
+      <c r="B1802" s="3"/>
+      <c r="C1802" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1802" s="3">
+        <v>6033011911</v>
+      </c>
+      <c r="E1802" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1802" s="3" t="s">
+        <v>710</v>
+      </c>
+      <c r="G1802" s="3" t="s">
+        <v>4537</v>
+      </c>
+      <c r="H1802" s="3"/>
+      <c r="I1802" s="3">
+        <v>76</v>
+      </c>
+      <c r="J1802" s="3">
+        <v>70</v>
+      </c>
+      <c r="K1802" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1802" s="3"/>
+      <c r="M1802" s="3"/>
+      <c r="N1802" s="3"/>
+    </row>
+    <row r="1803" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1803" s="3" t="s">
+        <v>4538</v>
+      </c>
+      <c r="B1803" s="3"/>
+      <c r="C1803" s="3">
+        <v>31</v>
+      </c>
+      <c r="D1803" s="3">
+        <v>6033245777</v>
+      </c>
+      <c r="E1803" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="F1803" s="3" t="s">
+        <v>1779</v>
+      </c>
+      <c r="G1803" s="3" t="s">
+        <v>4539</v>
+      </c>
+      <c r="H1803" s="3"/>
+      <c r="I1803" s="3">
+        <v>27</v>
+      </c>
+      <c r="J1803" s="3"/>
+      <c r="K1803" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1803" s="3"/>
+      <c r="M1803" s="3"/>
+      <c r="N1803" s="3"/>
+    </row>
+    <row r="1804" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1804" s="3" t="s">
+        <v>4540</v>
+      </c>
+      <c r="B1804" s="3"/>
+      <c r="C1804" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1804" s="3">
+        <v>6033599309</v>
+      </c>
+      <c r="E1804" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1804" s="3" t="s">
+        <v>1636</v>
+      </c>
+      <c r="G1804" s="3" t="s">
+        <v>4541</v>
+      </c>
+      <c r="H1804" s="3"/>
+      <c r="I1804" s="3">
+        <v>39</v>
+      </c>
+      <c r="J1804" s="3"/>
+      <c r="K1804" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1804" s="3"/>
+      <c r="M1804" s="3"/>
+      <c r="N1804" s="3"/>
+    </row>
+    <row r="1805" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1805" s="3" t="s">
+        <v>4542</v>
+      </c>
+      <c r="B1805" s="3"/>
+      <c r="C1805" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1805" s="3">
+        <v>6033615852</v>
+      </c>
+      <c r="E1805" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="F1805" s="3" t="s">
+        <v>693</v>
+      </c>
+      <c r="G1805" s="3" t="s">
+        <v>4543</v>
+      </c>
+      <c r="H1805" s="3"/>
+      <c r="I1805" s="3">
+        <v>21</v>
+      </c>
+      <c r="J1805" s="3"/>
+      <c r="K1805" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1805" s="3"/>
+      <c r="M1805" s="3"/>
+      <c r="N1805" s="3"/>
+    </row>
+    <row r="1806" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1806" s="3" t="s">
+        <v>4544</v>
+      </c>
+      <c r="B1806" s="3"/>
+      <c r="C1806" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1806" s="3">
+        <v>6033672954</v>
+      </c>
+      <c r="E1806" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1806" s="3" t="s">
+        <v>4545</v>
+      </c>
+      <c r="G1806" s="3" t="s">
+        <v>4546</v>
+      </c>
+      <c r="H1806" s="3"/>
+      <c r="I1806" s="3">
+        <v>34</v>
+      </c>
+      <c r="J1806" s="3"/>
+      <c r="K1806" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1806" s="3"/>
+      <c r="M1806" s="3"/>
+      <c r="N1806" s="3"/>
+    </row>
+    <row r="1807" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1807" s="3" t="s">
+        <v>4547</v>
+      </c>
+      <c r="B1807" s="3"/>
+      <c r="C1807" s="3">
+        <v>28</v>
+      </c>
+      <c r="D1807" s="3">
+        <v>6033675771</v>
+      </c>
+      <c r="E1807" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1807" s="3" t="s">
+        <v>4548</v>
+      </c>
+      <c r="G1807" s="3" t="s">
+        <v>4549</v>
+      </c>
+      <c r="H1807" s="3"/>
+      <c r="I1807" s="3">
+        <v>38</v>
+      </c>
+      <c r="J1807" s="3"/>
+      <c r="K1807" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1807" s="3"/>
+      <c r="M1807" s="3"/>
+      <c r="N1807" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>